<commit_message>
feat: regenerate sample workbook with Sections, Glossary, B/C items
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SampleChecklist.xlsx
+++ b/SampleChecklist.xlsx
@@ -9,6 +9,8 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checklist" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sections" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Glossary" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -414,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -529,7 +531,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Install counterweight safety gear and certify per EN81-20 §5.6.</t>
+          <t>Install counterweight safety gear and certify per EN81-20.</t>
         </is>
       </c>
     </row>
@@ -568,71 +570,63 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>A12</t>
+          <t>A13</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>PitToEarth: FALSE AND MaxFFLInt: &gt;11m</t>
+          <t>BuildingClass: "Class 9b" OR MaxFFLInt: &gt;=20</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Combined pit + travel safety review</t>
+          <t>Enhanced fire service controls</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>EN81-20</t>
+          <t>BCA</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Applies only when both conditions hold.</t>
+          <t>High-rise or assembly buildings need fire service lift controls.</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Perform a combined structural and travel safety assessment.</t>
+          <t>Provide fire service control switch and compliant signage.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>A13</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>BuildingClass: "Class 9b" OR MaxFFLInt: &gt;=20</t>
-        </is>
-      </c>
+          <t>B01</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Enhanced fire service controls</t>
+          <t>Pit structure designed for buffer impact loads</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>BCA</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>High-rise or assembly buildings need fire service lift controls.</t>
-        </is>
-      </c>
+          <t>AS1170</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Provide fire service control switch and compliant signage.</t>
+          <t>Confirm structural design accounts for buffer reaction forces.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>A14</t>
+          <t>B02</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -642,22 +636,78 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Provide accessible lift signage on every floor</t>
+          <t>Guide rail bracket spacing verified for travel</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>DDA</t>
+          <t>EN81-20</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Applies to taller installations.</t>
+          <t>Taller installations need verified bracket spacing.</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Install tactile/braille floor indicators at each landing.</t>
+          <t>Document guide-rail bracket spacing calculations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>C01</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Machine room power isolation provided</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>AS3000</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Install a lockable main switch for the lift supply.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>C02</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>PitToEarth: FALSE</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Earthing of car and well per wiring rules</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>AS3000</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Earthing continuity required where pit is not to solid earth.</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Measure and record earth continuity resistance.</t>
         </is>
       </c>
     </row>
@@ -814,4 +864,176 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Prefix</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Architectural</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Structural</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Electrical</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Term</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Meaning</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>AS3000</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>AS/NZS 3000 Wiring Rules — electrical installations standard. (sample text)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>AS1170</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>AS/NZS 1170 Structural design actions. (sample text)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>EN81-20</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>EN 81-20 — safety rules for the construction and installation of lifts. (sample text)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>BCA</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Building Code of Australia. (sample text)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>DDA</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Disability Discrimination Act — accessibility requirements. (sample text)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>State/local regulatory requirement. (sample text)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>RDM</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Reference Design Manual. (sample text)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: example images in a self-contained HTML report export
Add an optional "Example Image" column to the Checklist sheet (filename
in a local examples/ folder), parsed into item.exampleImage and
round-tripped through localStorage. Add an "Export report (with images)"
button that builds a portable HTML report of outstanding items per unit,
inlining each example image as a base64 data URI so clients get a single
self-contained file (the Excel export can't embed images).

Includes sample example images, regenerated SampleChecklist.xlsx with
the new column, README docs, and unit tests for optional-column parsing.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SampleChecklist.xlsx
+++ b/SampleChecklist.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -450,6 +450,11 @@
           <t>Example</t>
         </is>
       </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Example Image</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -478,6 +483,11 @@
           <t>Fit IP-rated enclosures and weather seals to the landing door head.</t>
         </is>
       </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>a08-weather-seal.svg</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -502,6 +512,7 @@
           <t>Provide a protected lobby between the lift and the dwelling entrance.</t>
         </is>
       </c>
+      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -534,6 +545,11 @@
           <t>Install counterweight safety gear and certify per EN81-20.</t>
         </is>
       </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>a10-cwt-safety.svg</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -566,6 +582,7 @@
           <t>Add emergency doors at max 11 m spacing along the well.</t>
         </is>
       </c>
+      <c r="G5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -598,6 +615,7 @@
           <t>Provide fire service control switch and compliant signage.</t>
         </is>
       </c>
+      <c r="G6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -622,6 +640,7 @@
           <t>Confirm structural design accounts for buffer reaction forces.</t>
         </is>
       </c>
+      <c r="G7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -654,6 +673,7 @@
           <t>Document guide-rail bracket spacing calculations.</t>
         </is>
       </c>
+      <c r="G8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -678,6 +698,7 @@
           <t>Install a lockable main switch for the lift supply.</t>
         </is>
       </c>
+      <c r="G9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -710,6 +731,7 @@
           <t>Measure and record earth continuity resistance.</t>
         </is>
       </c>
+      <c r="G10" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat: Excel export with embedded example photos (ExcelJS)
Vendor ExcelJS and replace the SheetJS unchecked-items export with one
that embeds each item's Example Image (PNG/JPG) directly into the row of
the .xlsx, so clients see the picture in Excel itself. Unsupported
formats (e.g. SVG) are noted in the cell rather than dropped silently.

Sample images converted SVG -> PNG (ExcelJS embeds raster only);
SampleChecklist.xlsx regenerated to reference the .png files. The HTML
report export still inlines any image type. README updated.

Verified end-to-end in headless Edge: export yields a valid xlsx with
xl/media/image1-2.png, oneCellAnchor drawings anchored to the A08/A10
rows, and correct content-types/rels wiring.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SampleChecklist.xlsx
+++ b/SampleChecklist.xlsx
@@ -485,7 +485,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>a08-weather-seal.svg</t>
+          <t>a08-weather-seal.png</t>
         </is>
       </c>
     </row>
@@ -547,7 +547,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>a10-cwt-safety.svg</t>
+          <t>a10-cwt-safety.png</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: single Example column holds prose OR an image filename
Drop the separate "Example Image" column. The Example cell is now
detected as an image when its value ends in an image extension
(.png/.jpg/.gif/.svg/.webp/.bmp); otherwise it is treated as prose
guidance. Internally still split into item.example (text) and
item.exampleImage (filename) so the HTML and Excel exports are unchanged.

Updates restore round-trip, sample workbook, unit tests, and README.
Verified end-to-end: Excel embeds the two image-cell pictures; the HTML
report shows images for image cells and "How to complete" prose for the
rest.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SampleChecklist.xlsx
+++ b/SampleChecklist.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -450,11 +450,6 @@
           <t>Example</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Example Image</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -480,11 +475,6 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Fit IP-rated enclosures and weather seals to the landing door head.</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
           <t>a08-weather-seal.png</t>
         </is>
       </c>
@@ -512,7 +502,6 @@
           <t>Provide a protected lobby between the lift and the dwelling entrance.</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -542,11 +531,6 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Install counterweight safety gear and certify per EN81-20.</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
           <t>a10-cwt-safety.png</t>
         </is>
       </c>
@@ -582,7 +566,6 @@
           <t>Add emergency doors at max 11 m spacing along the well.</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -615,7 +598,6 @@
           <t>Provide fire service control switch and compliant signage.</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -640,7 +622,6 @@
           <t>Confirm structural design accounts for buffer reaction forces.</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -673,7 +654,6 @@
           <t>Document guide-rail bracket spacing calculations.</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -698,7 +678,6 @@
           <t>Install a lockable main switch for the lift supply.</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -731,7 +710,6 @@
           <t>Measure and record earth continuity resistance.</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
docs: document the single-workbook setup and example links
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SampleChecklist.xlsx
+++ b/SampleChecklist.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -450,6 +450,11 @@
           <t>Example</t>
         </is>
       </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -478,6 +483,11 @@
           <t>a08-weather-seal.png</t>
         </is>
       </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>https://example.com/examples/a08-weather-seal.png</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -502,6 +512,7 @@
           <t>Provide a protected lobby between the lift and the dwelling entrance.</t>
         </is>
       </c>
+      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -534,6 +545,11 @@
           <t>a10-cwt-safety.png</t>
         </is>
       </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>https://example.com/examples/a10-cwt-safety.png</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -566,6 +582,7 @@
           <t>Add emergency doors at max 11 m spacing along the well.</t>
         </is>
       </c>
+      <c r="G5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -598,6 +615,7 @@
           <t>Provide fire service control switch and compliant signage.</t>
         </is>
       </c>
+      <c r="G6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -622,6 +640,7 @@
           <t>Confirm structural design accounts for buffer reaction forces.</t>
         </is>
       </c>
+      <c r="G7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -654,6 +673,7 @@
           <t>Document guide-rail bracket spacing calculations.</t>
         </is>
       </c>
+      <c r="G8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -678,6 +698,7 @@
           <t>Install a lockable main switch for the lift supply.</t>
         </is>
       </c>
+      <c r="G9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -710,6 +731,7 @@
           <t>Measure and record earth continuity resistance.</t>
         </is>
       </c>
+      <c r="G10" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>